<commit_message>
Update packages to remove null values from premise code & test on full dataset
</commit_message>
<xml_diff>
--- a/data/mo_codes.xlsx
+++ b/data/mo_codes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Career Goals\GitHub Projects\la-traffic-collision-analytics\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69FB53ED-1FAE-4352-8BA6-64F858B22BF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82E889C0-EE1C-4589-9645-1DE497D6480E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="781" uniqueCount="775">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="788" uniqueCount="775">
   <si>
     <t>mo_code</t>
   </si>
@@ -2708,7 +2708,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B780"/>
+  <dimension ref="A1:B787"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
@@ -8944,10 +8944,66 @@
       </c>
     </row>
     <row r="780" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A780" s="2">
+      <c r="A780">
         <v>3064</v>
       </c>
       <c r="B780" t="s">
+        <v>774</v>
+      </c>
+    </row>
+    <row r="781" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A781">
+        <v>3063</v>
+      </c>
+      <c r="B781" t="s">
+        <v>774</v>
+      </c>
+    </row>
+    <row r="782" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A782">
+        <v>2053</v>
+      </c>
+      <c r="B782" t="s">
+        <v>774</v>
+      </c>
+    </row>
+    <row r="783" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A783">
+        <v>1528</v>
+      </c>
+      <c r="B783" t="s">
+        <v>774</v>
+      </c>
+    </row>
+    <row r="784" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A784">
+        <v>1505</v>
+      </c>
+      <c r="B784" t="s">
+        <v>774</v>
+      </c>
+    </row>
+    <row r="785" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A785">
+        <v>1513</v>
+      </c>
+      <c r="B785" t="s">
+        <v>774</v>
+      </c>
+    </row>
+    <row r="786" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A786">
+        <v>2055</v>
+      </c>
+      <c r="B786" t="s">
+        <v>774</v>
+      </c>
+    </row>
+    <row r="787" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A787" s="2">
+        <v>3031</v>
+      </c>
+      <c r="B787" t="s">
         <v>774</v>
       </c>
     </row>

</xml_diff>